<commit_message>
Updates raw data cleaning
</commit_message>
<xml_diff>
--- a/0_Data/1_Household Data/1_Vietnam/3_Matching_Tables/Item_Categories_Concordance_Vietnam.xlsx
+++ b/0_Data/1_Household Data/1_Vietnam/3_Matching_Tables/Item_Categories_Concordance_Vietnam.xlsx
@@ -14,7 +14,7 @@
   <sheets>
     <sheet name="Item_Vietnam" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="162913" concurrentCalc="0"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -54,7 +54,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -69,19 +69,19 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -113,7 +113,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -403,8 +403,8 @@
     <col min="7" max="12" width="4.453125" bestFit="1" customWidth="1"/>
     <col min="13" max="14" width="5.36328125" bestFit="1" customWidth="1"/>
     <col min="15" max="27" width="3.54296875" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="4.453125" bestFit="1" customWidth="1"/>
-    <col min="29" max="39" width="3.54296875" bestFit="1" customWidth="1"/>
+    <col min="28" max="29" width="4.453125" bestFit="1" customWidth="1"/>
+    <col min="30" max="39" width="3.54296875" bestFit="1" customWidth="1"/>
     <col min="40" max="42" width="4.453125" bestFit="1" customWidth="1"/>
     <col min="43" max="75" width="5.36328125" bestFit="1" customWidth="1"/>
     <col min="76" max="138" width="10.90625" customWidth="1"/>
@@ -414,188 +414,228 @@
       <c r="A1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B1" s="3">
+      <c r="B1" s="1">
         <v>101</v>
       </c>
-      <c r="C1" s="3">
+      <c r="C1" s="1">
         <v>102</v>
       </c>
-      <c r="D1" s="3">
+      <c r="D1" s="1">
         <v>103</v>
       </c>
-      <c r="E1" s="3">
+      <c r="E1" s="1">
         <v>104</v>
       </c>
-      <c r="F1" s="3">
+      <c r="F1" s="1">
         <v>105</v>
       </c>
-      <c r="G1" s="3">
+      <c r="G1" s="1">
         <v>106</v>
       </c>
-      <c r="H1" s="3">
+      <c r="H1" s="1">
         <v>107</v>
       </c>
-      <c r="I1" s="3">
+      <c r="I1" s="1">
         <v>108</v>
       </c>
-      <c r="J1" s="3">
+      <c r="J1" s="1">
         <v>109</v>
       </c>
-      <c r="K1" s="3">
+      <c r="K1" s="1">
         <v>110</v>
       </c>
-      <c r="L1" s="3">
+      <c r="L1" s="1">
         <v>111</v>
       </c>
-      <c r="M1" s="3">
+      <c r="M1" s="1">
         <v>112</v>
       </c>
-      <c r="N1" s="3">
+      <c r="N1" s="1">
         <v>113</v>
       </c>
-      <c r="O1" s="3">
+      <c r="O1" s="1">
         <v>114</v>
       </c>
-      <c r="P1" s="3">
+      <c r="P1" s="1">
         <v>115</v>
       </c>
-      <c r="Q1" s="3">
+      <c r="Q1" s="1">
         <v>116</v>
       </c>
-      <c r="R1" s="3">
+      <c r="R1" s="1">
         <v>117</v>
       </c>
-      <c r="S1" s="3">
+      <c r="S1" s="1">
         <v>118</v>
       </c>
-      <c r="T1" s="3">
+      <c r="T1" s="1">
         <v>119</v>
       </c>
-      <c r="U1" s="3">
+      <c r="U1" s="1">
         <v>120</v>
       </c>
-      <c r="V1" s="3">
+      <c r="V1" s="1">
         <v>121</v>
       </c>
-      <c r="W1" s="3">
+      <c r="W1" s="1">
         <v>122</v>
       </c>
-      <c r="X1" s="3">
+      <c r="X1" s="1">
         <v>123</v>
       </c>
-      <c r="Y1" s="3">
+      <c r="Y1" s="1">
         <v>124</v>
       </c>
-      <c r="Z1" s="3">
+      <c r="Z1" s="1">
         <v>125</v>
       </c>
-      <c r="AA1" s="3">
+      <c r="AA1" s="1">
         <v>126</v>
       </c>
-      <c r="AB1" s="3">
+      <c r="AB1" s="1">
         <v>127</v>
       </c>
-      <c r="AC1" s="3">
+      <c r="AC1" s="1">
         <v>128</v>
       </c>
-      <c r="AD1" s="3">
+      <c r="AD1" s="1">
         <v>129</v>
       </c>
-      <c r="AE1" s="3">
+      <c r="AE1" s="1">
         <v>130</v>
       </c>
-      <c r="AF1" s="3">
+      <c r="AF1" s="1">
         <v>131</v>
       </c>
-      <c r="AG1" s="3">
+      <c r="AG1" s="1">
         <v>132</v>
       </c>
-      <c r="AH1" s="3">
+      <c r="AH1" s="1">
         <v>133</v>
       </c>
-      <c r="AI1" s="3">
+      <c r="AI1" s="1">
         <v>134</v>
       </c>
-      <c r="AJ1" s="3">
+      <c r="AJ1" s="1">
         <v>135</v>
       </c>
-      <c r="AK1" s="3">
+      <c r="AK1" s="1">
+        <v>136</v>
+      </c>
+      <c r="AL1" s="1">
         <v>137</v>
       </c>
-      <c r="AL1" s="3">
+      <c r="AM1" s="1">
         <v>138</v>
       </c>
-      <c r="AM1" s="3">
+      <c r="AN1" s="1">
         <v>139</v>
       </c>
-      <c r="AN1" s="3">
+      <c r="AO1" s="1">
         <v>140</v>
       </c>
-      <c r="AO1" s="3">
+      <c r="AP1" s="1">
         <v>141</v>
       </c>
-      <c r="AP1" s="3">
+      <c r="AQ1" s="1">
         <v>142</v>
       </c>
-      <c r="AQ1" s="3">
+      <c r="AR1" s="1">
         <v>143</v>
       </c>
-      <c r="AR1" s="3">
+      <c r="AS1" s="1">
         <v>144</v>
       </c>
-      <c r="AS1" s="3">
+      <c r="AT1" s="1">
         <v>145</v>
       </c>
-      <c r="AT1" s="3">
+      <c r="AU1" s="1">
         <v>146</v>
       </c>
-      <c r="AU1" s="3">
+      <c r="AV1" s="1">
         <v>147</v>
       </c>
-      <c r="AV1" s="3">
+      <c r="AW1" s="1">
         <v>148</v>
       </c>
-      <c r="AW1" s="3">
+      <c r="AX1" s="1">
         <v>149</v>
       </c>
-      <c r="AX1" s="3">
+      <c r="AY1" s="1">
         <v>150</v>
       </c>
-      <c r="AY1" s="3">
-        <v>151</v>
-      </c>
-      <c r="AZ1" s="3">
-        <v>152</v>
-      </c>
-      <c r="BA1" s="3">
-        <v>153</v>
-      </c>
-      <c r="BB1" s="3">
-        <v>154</v>
+      <c r="AZ1" s="1">
+        <v>10100</v>
+      </c>
+      <c r="BA1" s="1">
+        <v>10200</v>
+      </c>
+      <c r="BB1" s="1">
+        <v>11000</v>
       </c>
       <c r="BC1" s="1">
-        <v>136</v>
-      </c>
-      <c r="BD1" s="1"/>
-      <c r="BE1" s="1"/>
-      <c r="BF1" s="1"/>
-      <c r="BG1" s="1"/>
-      <c r="BH1" s="1"/>
-      <c r="BI1" s="1"/>
-      <c r="BJ1" s="1"/>
-      <c r="BK1" s="1"/>
-      <c r="BL1" s="1"/>
-      <c r="BM1" s="1"/>
-      <c r="BN1" s="1"/>
-      <c r="BO1" s="1"/>
-      <c r="BP1" s="1"/>
-      <c r="BQ1" s="1"/>
-      <c r="BR1" s="1"/>
-      <c r="BS1" s="1"/>
-      <c r="BT1" s="1"/>
-      <c r="BU1" s="1"/>
-      <c r="BV1" s="1"/>
-      <c r="BW1" s="1"/>
+        <v>11100</v>
+      </c>
+      <c r="BD1" s="1">
+        <v>11200</v>
+      </c>
+      <c r="BE1" s="1">
+        <v>11300</v>
+      </c>
+      <c r="BF1" s="1">
+        <v>11400</v>
+      </c>
+      <c r="BG1" s="1">
+        <v>11500</v>
+      </c>
+      <c r="BH1" s="1">
+        <v>11600</v>
+      </c>
+      <c r="BI1" s="1">
+        <v>11800</v>
+      </c>
+      <c r="BJ1" s="1">
+        <v>12000</v>
+      </c>
+      <c r="BK1" s="1">
+        <v>12100</v>
+      </c>
+      <c r="BL1" s="1">
+        <v>12400</v>
+      </c>
+      <c r="BM1" s="1">
+        <v>13400</v>
+      </c>
+      <c r="BN1" s="1">
+        <v>13900</v>
+      </c>
+      <c r="BO1" s="1">
+        <v>14000</v>
+      </c>
+      <c r="BP1" s="1">
+        <v>14400</v>
+      </c>
+      <c r="BQ1" s="1">
+        <v>14500</v>
+      </c>
+      <c r="BR1" s="1">
+        <v>14600</v>
+      </c>
+      <c r="BS1" s="1">
+        <v>14800</v>
+      </c>
+      <c r="BT1" s="1">
+        <v>15000</v>
+      </c>
+      <c r="BU1" s="1">
+        <v>15100</v>
+      </c>
+      <c r="BV1" s="1">
+        <v>15300</v>
+      </c>
+      <c r="BW1" s="1">
+        <v>15400</v>
+      </c>
       <c r="BX1" s="1"/>
       <c r="BY1" s="1"/>
       <c r="BZ1" s="1"/>
@@ -664,45 +704,43 @@
       <c r="A2" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="3">
+      <c r="B2" s="1">
+        <v>1024</v>
+      </c>
+      <c r="C2" s="1">
         <v>202</v>
       </c>
-      <c r="C2" s="3">
+      <c r="D2" s="1">
         <v>203</v>
       </c>
-      <c r="D2" s="3">
+      <c r="E2" s="1">
         <v>204</v>
       </c>
-      <c r="E2" s="3">
+      <c r="F2" s="1">
         <v>205</v>
       </c>
-      <c r="F2" s="3">
+      <c r="G2" s="1">
         <v>206</v>
       </c>
-      <c r="G2" s="3">
+      <c r="H2" s="1">
         <v>207</v>
       </c>
-      <c r="H2" s="3">
+      <c r="I2" s="1">
         <v>208</v>
       </c>
-      <c r="I2" s="3">
+      <c r="J2" s="1">
         <v>209</v>
       </c>
-      <c r="J2" s="3">
+      <c r="K2" s="1">
         <v>210</v>
       </c>
-      <c r="K2" s="3">
+      <c r="L2" s="1">
         <v>211</v>
       </c>
-      <c r="L2" s="3">
+      <c r="M2" s="1">
         <v>212</v>
       </c>
-      <c r="M2" s="3">
-        <v>213</v>
-      </c>
-      <c r="N2" s="3">
-        <v>1024</v>
-      </c>
+      <c r="N2" s="1"/>
       <c r="O2" s="1"/>
       <c r="P2" s="1"/>
       <c r="Q2" s="1"/>
@@ -832,233 +870,237 @@
       <c r="A3" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="3">
+      <c r="B3" s="1">
+        <v>151</v>
+      </c>
+      <c r="C3" s="1">
+        <v>152</v>
+      </c>
+      <c r="D3" s="1">
+        <v>214</v>
+      </c>
+      <c r="E3" s="1">
+        <v>215</v>
+      </c>
+      <c r="F3" s="1">
+        <v>216</v>
+      </c>
+      <c r="G3" s="1">
+        <v>217</v>
+      </c>
+      <c r="H3" s="1">
+        <v>218</v>
+      </c>
+      <c r="I3" s="1">
+        <v>219</v>
+      </c>
+      <c r="J3" s="1">
+        <v>220</v>
+      </c>
+      <c r="K3" s="1">
+        <v>221</v>
+      </c>
+      <c r="L3" s="1">
+        <v>222</v>
+      </c>
+      <c r="M3" s="1">
+        <v>223</v>
+      </c>
+      <c r="N3" s="1">
+        <v>224</v>
+      </c>
+      <c r="O3" s="1">
+        <v>226</v>
+      </c>
+      <c r="P3" s="1">
+        <v>227</v>
+      </c>
+      <c r="Q3" s="1">
+        <v>301</v>
+      </c>
+      <c r="R3" s="1">
+        <v>302</v>
+      </c>
+      <c r="S3" s="1">
+        <v>303</v>
+      </c>
+      <c r="T3" s="1">
+        <v>304</v>
+      </c>
+      <c r="U3" s="1">
+        <v>305</v>
+      </c>
+      <c r="V3" s="1">
+        <v>306</v>
+      </c>
+      <c r="W3" s="1">
+        <v>308</v>
+      </c>
+      <c r="X3" s="1">
+        <v>309</v>
+      </c>
+      <c r="Y3" s="1">
+        <v>310</v>
+      </c>
+      <c r="Z3" s="1">
+        <v>311</v>
+      </c>
+      <c r="AA3" s="1">
+        <v>312</v>
+      </c>
+      <c r="AB3" s="1">
+        <v>313</v>
+      </c>
+      <c r="AC3" s="1">
+        <v>314</v>
+      </c>
+      <c r="AD3" s="1">
+        <v>315</v>
+      </c>
+      <c r="AE3" s="1">
+        <v>316</v>
+      </c>
+      <c r="AF3" s="1">
+        <v>317</v>
+      </c>
+      <c r="AG3" s="1">
+        <v>318</v>
+      </c>
+      <c r="AH3" s="1">
+        <v>322</v>
+      </c>
+      <c r="AI3" s="1">
+        <v>323</v>
+      </c>
+      <c r="AJ3" s="1">
+        <v>324</v>
+      </c>
+      <c r="AK3" s="1">
+        <v>325</v>
+      </c>
+      <c r="AL3" s="1">
+        <v>326</v>
+      </c>
+      <c r="AM3" s="1">
+        <v>333</v>
+      </c>
+      <c r="AN3" s="1">
+        <v>7</v>
+      </c>
+      <c r="AO3" s="1">
+        <v>8</v>
+      </c>
+      <c r="AP3" s="1">
+        <v>9</v>
+      </c>
+      <c r="AQ3" s="1">
+        <v>11</v>
+      </c>
+      <c r="AR3" s="1">
+        <v>12</v>
+      </c>
+      <c r="AS3" s="1">
+        <v>13</v>
+      </c>
+      <c r="AT3" s="1">
+        <v>14</v>
+      </c>
+      <c r="AU3" s="1">
+        <v>15</v>
+      </c>
+      <c r="AV3" s="1">
+        <v>16</v>
+      </c>
+      <c r="AW3" s="1">
+        <v>17</v>
+      </c>
+      <c r="AX3" s="1">
+        <v>18</v>
+      </c>
+      <c r="AY3" s="1">
+        <v>19</v>
+      </c>
+      <c r="AZ3" s="1">
+        <v>20</v>
+      </c>
+      <c r="BA3" s="1">
+        <v>21</v>
+      </c>
+      <c r="BB3" s="1">
+        <v>22</v>
+      </c>
+      <c r="BC3" s="1">
+        <v>23</v>
+      </c>
+      <c r="BD3" s="1">
+        <v>24</v>
+      </c>
+      <c r="BE3" s="1">
+        <v>25</v>
+      </c>
+      <c r="BF3" s="1">
+        <v>26</v>
+      </c>
+      <c r="BG3" s="1">
+        <v>27</v>
+      </c>
+      <c r="BH3" s="1">
+        <v>28</v>
+      </c>
+      <c r="BI3" s="1">
+        <v>29</v>
+      </c>
+      <c r="BJ3" s="1">
+        <v>30</v>
+      </c>
+      <c r="BK3" s="1">
+        <v>31</v>
+      </c>
+      <c r="BL3" s="1">
+        <v>32</v>
+      </c>
+      <c r="BM3" s="1">
+        <v>33</v>
+      </c>
+      <c r="BN3" s="1">
+        <v>34</v>
+      </c>
+      <c r="BO3" s="1">
+        <v>35</v>
+      </c>
+      <c r="BP3" s="1">
+        <v>36</v>
+      </c>
+      <c r="BQ3" s="1">
+        <v>319</v>
+      </c>
+      <c r="BR3" s="1">
         <v>1</v>
       </c>
-      <c r="C3" s="3">
+      <c r="BS3" s="1">
         <v>2</v>
       </c>
-      <c r="D3" s="3">
+      <c r="BT3" s="1">
         <v>3</v>
       </c>
-      <c r="E3" s="3">
+      <c r="BU3" s="1">
         <v>4</v>
       </c>
-      <c r="F3" s="3">
+      <c r="BV3" s="1">
         <v>5</v>
       </c>
-      <c r="G3" s="3">
+      <c r="BW3" s="1">
         <v>6</v>
       </c>
-      <c r="H3" s="3">
-        <v>7</v>
-      </c>
-      <c r="I3" s="3">
-        <v>8</v>
-      </c>
-      <c r="J3" s="3">
-        <v>9</v>
-      </c>
-      <c r="K3" s="3">
-        <v>10</v>
-      </c>
-      <c r="L3" s="3">
-        <v>11</v>
-      </c>
-      <c r="M3" s="3">
-        <v>12</v>
-      </c>
-      <c r="N3" s="3">
-        <v>13</v>
-      </c>
-      <c r="O3" s="3">
-        <v>14</v>
-      </c>
-      <c r="P3" s="3">
-        <v>15</v>
-      </c>
-      <c r="Q3" s="3">
-        <v>16</v>
-      </c>
-      <c r="R3" s="3">
-        <v>17</v>
-      </c>
-      <c r="S3" s="3">
-        <v>18</v>
-      </c>
-      <c r="T3" s="3">
-        <v>19</v>
-      </c>
-      <c r="U3" s="3">
-        <v>20</v>
-      </c>
-      <c r="V3" s="3">
-        <v>21</v>
-      </c>
-      <c r="W3" s="3">
-        <v>22</v>
-      </c>
-      <c r="X3" s="3">
-        <v>23</v>
-      </c>
-      <c r="Y3" s="3">
-        <v>24</v>
-      </c>
-      <c r="Z3" s="3">
-        <v>25</v>
-      </c>
-      <c r="AA3" s="3">
-        <v>26</v>
-      </c>
-      <c r="AB3" s="3">
-        <v>27</v>
-      </c>
-      <c r="AC3" s="3">
-        <v>28</v>
-      </c>
-      <c r="AD3" s="3">
-        <v>29</v>
-      </c>
-      <c r="AE3" s="3">
-        <v>30</v>
-      </c>
-      <c r="AF3" s="3">
-        <v>31</v>
-      </c>
-      <c r="AG3" s="3">
-        <v>32</v>
-      </c>
-      <c r="AH3" s="3">
-        <v>33</v>
-      </c>
-      <c r="AI3" s="3">
-        <v>34</v>
-      </c>
-      <c r="AJ3" s="3">
-        <v>35</v>
-      </c>
-      <c r="AK3" s="3">
-        <v>37</v>
-      </c>
-      <c r="AL3" s="3">
+      <c r="BX3" s="3">
         <v>42</v>
       </c>
-      <c r="AM3" s="3">
+      <c r="BY3" s="3">
         <v>43</v>
       </c>
-      <c r="AN3" s="3">
-        <v>215</v>
-      </c>
-      <c r="AO3" s="3">
-        <v>216</v>
-      </c>
-      <c r="AP3" s="3">
-        <v>217</v>
-      </c>
-      <c r="AQ3" s="3">
-        <v>218</v>
-      </c>
-      <c r="AR3" s="3">
-        <v>219</v>
-      </c>
-      <c r="AS3" s="3">
-        <v>220</v>
-      </c>
-      <c r="AT3" s="3">
-        <v>221</v>
-      </c>
-      <c r="AU3" s="3">
-        <v>222</v>
-      </c>
-      <c r="AV3" s="3">
-        <v>223</v>
-      </c>
-      <c r="AW3" s="3">
-        <v>224</v>
-      </c>
-      <c r="AX3" s="3">
-        <v>225</v>
-      </c>
-      <c r="AY3" s="3">
-        <v>226</v>
-      </c>
-      <c r="AZ3" s="3">
-        <v>227</v>
-      </c>
-      <c r="BA3" s="3">
-        <v>301</v>
-      </c>
-      <c r="BB3" s="3">
-        <v>302</v>
-      </c>
-      <c r="BC3" s="3">
-        <v>303</v>
-      </c>
-      <c r="BD3" s="3">
-        <v>304</v>
-      </c>
-      <c r="BE3" s="3">
-        <v>305</v>
-      </c>
-      <c r="BF3" s="3">
-        <v>306</v>
-      </c>
-      <c r="BG3" s="3">
-        <v>308</v>
-      </c>
-      <c r="BH3" s="3">
-        <v>309</v>
-      </c>
-      <c r="BI3" s="3">
-        <v>310</v>
-      </c>
-      <c r="BJ3" s="3">
-        <v>311</v>
-      </c>
-      <c r="BK3" s="3">
-        <v>312</v>
-      </c>
-      <c r="BL3" s="3">
-        <v>313</v>
-      </c>
-      <c r="BM3" s="3">
-        <v>314</v>
-      </c>
-      <c r="BN3" s="3">
-        <v>315</v>
-      </c>
-      <c r="BO3" s="3">
-        <v>316</v>
-      </c>
-      <c r="BP3" s="3">
-        <v>317</v>
-      </c>
-      <c r="BQ3" s="3">
-        <v>318</v>
-      </c>
-      <c r="BR3" s="3">
-        <v>319</v>
-      </c>
-      <c r="BS3" s="3">
-        <v>322</v>
-      </c>
-      <c r="BT3" s="3">
-        <v>323</v>
-      </c>
-      <c r="BU3" s="3">
-        <v>324</v>
-      </c>
-      <c r="BV3" s="3">
-        <v>325</v>
-      </c>
-      <c r="BW3" s="3">
-        <v>333</v>
-      </c>
-      <c r="BX3" s="1">
+      <c r="BZ3" s="3">
         <v>44</v>
       </c>
-      <c r="BY3" s="1"/>
-      <c r="BZ3" s="1"/>
       <c r="CA3" s="1"/>
       <c r="CB3" s="1"/>
       <c r="CC3" s="1"/>
@@ -1124,107 +1166,109 @@
       <c r="A4" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="3">
+      <c r="B4" s="1">
+        <v>1008</v>
+      </c>
+      <c r="C4" s="1"/>
+      <c r="D4" s="1">
+        <v>1020</v>
+      </c>
+      <c r="E4" s="1">
+        <v>1026</v>
+      </c>
+      <c r="F4" s="1">
+        <v>153</v>
+      </c>
+      <c r="G4" s="1">
+        <v>201</v>
+      </c>
+      <c r="H4" s="1">
+        <v>213</v>
+      </c>
+      <c r="I4" s="1">
+        <v>225</v>
+      </c>
+      <c r="J4" s="1">
+        <v>307</v>
+      </c>
+      <c r="K4" s="1">
+        <v>320</v>
+      </c>
+      <c r="L4" s="1">
+        <v>327</v>
+      </c>
+      <c r="M4" s="1">
+        <v>328</v>
+      </c>
+      <c r="N4" s="1">
+        <v>329</v>
+      </c>
+      <c r="O4" s="1">
+        <v>330</v>
+      </c>
+      <c r="P4" s="1">
+        <v>331</v>
+      </c>
+      <c r="Q4" s="1">
+        <v>332</v>
+      </c>
+      <c r="R4" s="1">
+        <v>334</v>
+      </c>
+      <c r="S4" s="1">
+        <v>335</v>
+      </c>
+      <c r="T4" s="1">
+        <v>400</v>
+      </c>
+      <c r="U4" s="1">
+        <v>401</v>
+      </c>
+      <c r="V4" s="1">
+        <v>402</v>
+      </c>
+      <c r="W4" s="1">
+        <v>403</v>
+      </c>
+      <c r="X4" s="1">
+        <v>404</v>
+      </c>
+      <c r="Y4" s="1">
+        <v>405</v>
+      </c>
+      <c r="Z4" s="1">
+        <v>406</v>
+      </c>
+      <c r="AA4" s="1">
+        <v>407</v>
+      </c>
+      <c r="AB4" s="1">
+        <v>1530</v>
+      </c>
+      <c r="AC4" s="1">
+        <v>1014</v>
+      </c>
+      <c r="AD4" s="1">
+        <v>321</v>
+      </c>
+      <c r="AE4" s="3">
         <v>38</v>
       </c>
-      <c r="C4" s="3">
+      <c r="AF4" s="3">
         <v>39</v>
       </c>
-      <c r="D4" s="3">
+      <c r="AG4" s="3">
         <v>40</v>
       </c>
-      <c r="E4" s="3">
+      <c r="AH4" s="3">
         <v>41</v>
       </c>
-      <c r="F4" s="3">
+      <c r="AI4" s="3">
         <v>45</v>
       </c>
-      <c r="G4" s="3">
+      <c r="AJ4" s="3">
         <v>46</v>
       </c>
-      <c r="H4" s="3">
-        <v>201</v>
-      </c>
-      <c r="I4" s="3">
-        <v>214</v>
-      </c>
-      <c r="J4" s="3">
-        <v>228</v>
-      </c>
-      <c r="K4" s="3">
-        <v>307</v>
-      </c>
-      <c r="L4" s="3">
-        <v>320</v>
-      </c>
-      <c r="M4" s="3">
-        <v>321</v>
-      </c>
-      <c r="N4" s="3">
-        <v>326</v>
-      </c>
-      <c r="O4" s="3">
-        <v>327</v>
-      </c>
-      <c r="P4" s="3">
-        <v>328</v>
-      </c>
-      <c r="Q4" s="3">
-        <v>329</v>
-      </c>
-      <c r="R4" s="3">
-        <v>330</v>
-      </c>
-      <c r="S4" s="3">
-        <v>331</v>
-      </c>
-      <c r="T4" s="3">
-        <v>332</v>
-      </c>
-      <c r="U4" s="3">
-        <v>334</v>
-      </c>
-      <c r="V4" s="3">
-        <v>335</v>
-      </c>
-      <c r="W4" s="3">
-        <v>336</v>
-      </c>
-      <c r="X4" s="3">
-        <v>400</v>
-      </c>
-      <c r="Y4" s="3">
-        <v>401</v>
-      </c>
-      <c r="Z4" s="3">
-        <v>402</v>
-      </c>
-      <c r="AA4" s="3">
-        <v>404</v>
-      </c>
-      <c r="AB4" s="3">
-        <v>405</v>
-      </c>
-      <c r="AC4" s="3">
-        <v>406</v>
-      </c>
-      <c r="AD4" s="3">
-        <v>407</v>
-      </c>
-      <c r="AE4" s="3">
-        <v>1008</v>
-      </c>
-      <c r="AF4" s="3">
-        <v>1014</v>
-      </c>
-      <c r="AG4" s="3">
-        <v>1020</v>
-      </c>
-      <c r="AH4" s="3">
-        <v>1026</v>
-      </c>
-      <c r="AI4" s="1"/>
-      <c r="AJ4" s="1"/>
       <c r="AK4" s="1"/>
       <c r="AL4" s="1"/>
       <c r="AM4" s="1"/>
@@ -1332,15 +1376,21 @@
       <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="3">
-        <v>229</v>
-      </c>
-      <c r="C5" s="3">
+      <c r="B5" s="1">
+        <v>154</v>
+      </c>
+      <c r="C5" s="1">
+        <v>228</v>
+      </c>
+      <c r="D5" s="1">
+        <v>336</v>
+      </c>
+      <c r="E5" s="1">
         <v>408</v>
       </c>
-      <c r="D5" s="1"/>
-      <c r="E5" s="1"/>
-      <c r="F5" s="1"/>
+      <c r="F5" s="1">
+        <v>37</v>
+      </c>
       <c r="G5" s="1"/>
       <c r="H5" s="1"/>
       <c r="I5" s="1"/>
@@ -1478,21 +1528,45 @@
       <c r="A6" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B6" s="3">
-        <v>403</v>
-      </c>
-      <c r="C6" s="1"/>
-      <c r="D6" s="1"/>
-      <c r="E6" s="1"/>
-      <c r="F6" s="1"/>
-      <c r="G6" s="1"/>
-      <c r="H6" s="1"/>
-      <c r="I6" s="1"/>
-      <c r="J6" s="1"/>
-      <c r="K6" s="1"/>
-      <c r="L6" s="1"/>
-      <c r="M6" s="1"/>
-      <c r="N6" s="1"/>
+      <c r="B6" s="1">
+        <v>1011</v>
+      </c>
+      <c r="C6" s="1">
+        <v>1012</v>
+      </c>
+      <c r="D6" s="1">
+        <v>1171</v>
+      </c>
+      <c r="E6" s="1">
+        <v>1172</v>
+      </c>
+      <c r="F6" s="1">
+        <v>1181</v>
+      </c>
+      <c r="G6" s="1">
+        <v>1182</v>
+      </c>
+      <c r="H6" s="1">
+        <v>1411</v>
+      </c>
+      <c r="I6" s="1">
+        <v>1412</v>
+      </c>
+      <c r="J6" s="1">
+        <v>1531</v>
+      </c>
+      <c r="K6" s="1">
+        <v>1532</v>
+      </c>
+      <c r="L6" s="1">
+        <v>1533</v>
+      </c>
+      <c r="M6" s="1">
+        <v>11810</v>
+      </c>
+      <c r="N6" s="1">
+        <v>11820</v>
+      </c>
       <c r="O6" s="1"/>
       <c r="P6" s="1"/>
       <c r="Q6" s="1"/>

</xml_diff>